<commit_message>
Brief 91b P1: brief landing + EP-flag-rename rider + session reconcile
- Land 91b brief at docs/briefs/active/91b_cost_plan_editor.md.
- Rider: in the HIEX report export, soften "EP-validated ✓" →
  "EP-checked — see Table 3" where the EP EUI cross-check diverges
  |Δ%| > 25 (Chris's chosen metric, 2026-07-08). The brief's
  "(currently 3.3)" parenthetical was stale; the |EUI Δ%|>25 rule
  trips 2.2, 3.3, 3.4, 3.5. CSV + XLSX regenerated — only those 4
  flag cells changed, all other data byte-identical.
- Reconcile current.md + STATUS.md: 91b now the active brief;
  95 (PR #2) and 96 (PR #3) marked merged to main.

Zero physics — --fixture anchor EUI 132.6 unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/report/HIEX_intervention_metrics.xlsx
+++ b/docs/report/HIEX_intervention_metrics.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t xml:space="preserve">EP-validated ✓ </t>
+          <t xml:space="preserve">EP-checked — see Table 3 </t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t xml:space="preserve">EP-validated ✓ </t>
+          <t xml:space="preserve">EP-checked — see Table 3 </t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t xml:space="preserve">EP-validated ✓ </t>
+          <t xml:space="preserve">EP-checked — see Table 3 </t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t xml:space="preserve">EP-validated ✓ </t>
+          <t xml:space="preserve">EP-checked — see Table 3 </t>
         </is>
       </c>
       <c r="R15" t="inlineStr">

</xml_diff>